<commit_message>
V4.1b pre-review fixes: scrollable prayer list (8 selectable), era card outside the list, panel to y=640, compact prayer cards, larger god/mode card text, first council in the first autumn, opening forecast refit; sheet2code tool (NPC trial, data kept out of the build)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/輪廻の天秤_仕様書_規格書_v0.9.xlsx
+++ b/docs/輪廻の天秤_仕様書_規格書_v0.9.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1596" uniqueCount="1162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1602" uniqueCount="1168">
   <si>
     <t>《輪廻の天秤》仕様書 / 《輪迴之天秤》規格書</t>
   </si>
@@ -3200,6 +3200,15 @@
     <t>總指示書第一部 A/B/C 與視覺總指示書第二部（開頭畫面）。工作表 18。V4.2 在視覺總指示書第一部（點陣 100%）完成後重做。</t>
   </si>
   <si>
+    <t>v0.9b / V4.1b</t>
+  </si>
+  <si>
+    <t>預審 §2：祈りリストがスクロール（8件すべて選択可）、時代の兆しはリストの外、右パネルは y=62〜640、祈りカードは1行（選ぶと展開）、神格・モードカードの文字 18〜22px、最初の評定会は1年目の秋、開局の「その時」予測（engaged 23局で各区間の誤差 ≦13pt）。</t>
+  </si>
+  <si>
+    <t>預審 §2：祈禱清單可捲動（8 個都能選）、時代徵兆放在清單外、右側面板 y=62～640、祈禱卡精簡成一行（選取後展開）、神格與模式卡文字 18～22px、第一次評定會延到第 1 年秋天、開局「屆時」預估（engaged 23 局各區間誤差 ≦13pt）。</t>
+  </si>
+  <si>
     <t>V4 攻防・評定会 / V4 攻防與評定會</t>
   </si>
   <si>
@@ -3519,6 +3528,15 @@
   </si>
   <si>
     <t>v4_sim / card_click（×1・×16 各10回）/ pray_two / ui_cover（通常29%・たたむ9%・U 4%）/ ruins_sim（2.00/4.00/6.00日）/ ruins_ui / title_flow / title_pixel / smoke / tut_v41 / v4_ui / story_check 4/60（V4.1 と同じ）/ lang / soak 20/20</t>
+  </si>
+  <si>
+    <t>V4.1b 修正</t>
+  </si>
+  <si>
+    <t>祈りリストのスクロール、時代の兆しの位置、右パネルの高さ、1行の祈りカード、カードの文字サイズ、評定会の時期（1年目の秋）、開局予測の再調整。</t>
+  </si>
+  <si>
+    <t>祈禱清單捲動、時代徵兆位置、右側面板高度、一行祈禱卡、卡片字級、評定會時機（第 1 年秋天）、開局預估重新校準。</t>
   </si>
 </sst>
 </file>
@@ -7196,7 +7214,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -7349,6 +7367,17 @@
       </c>
       <c r="C15" s="11" t="s">
         <v>1054</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>1057</v>
       </c>
     </row>
   </sheetData>
@@ -7368,24 +7397,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1055</v>
+        <v>1058</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7401,156 +7430,156 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1057</v>
+        <v>1060</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1058</v>
+        <v>1061</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1060</v>
+        <v>1063</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1061</v>
+        <v>1064</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1062</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1063</v>
+        <v>1066</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1064</v>
+        <v>1067</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1065</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1066</v>
+        <v>1069</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1067</v>
+        <v>1070</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1069</v>
+        <v>1072</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1070</v>
+        <v>1073</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1071</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1072</v>
+        <v>1075</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1073</v>
+        <v>1076</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1074</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1077</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1079</v>
+        <v>1082</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1080</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1083</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1085</v>
+        <v>1088</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1086</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>1087</v>
+        <v>1090</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>1092</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>1093</v>
+        <v>1096</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>1094</v>
+        <v>1097</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>1095</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>1098</v>
+        <v>1101</v>
       </c>
     </row>
   </sheetData>
@@ -7570,24 +7599,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7603,123 +7632,123 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1100</v>
+        <v>1103</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
     </row>
   </sheetData>
@@ -7862,7 +7891,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -7871,24 +7900,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7904,117 +7933,128 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1139</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1154</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1155</v>
+        <v>1158</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1159</v>
+        <v>1162</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1160</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1161</v>
+        <v>1164</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1161</v>
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>1167</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Spec v0.9c: changelog for the visual 100% integration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/輪廻の天秤_仕様書_規格書_v0.9.xlsx
+++ b/docs/輪廻の天秤_仕様書_規格書_v0.9.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1602" uniqueCount="1168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="1174">
   <si>
     <t>《輪廻の天秤》仕様書 / 《輪迴之天秤》規格書</t>
   </si>
@@ -3209,6 +3209,15 @@
     <t>預審 §2：祈禱清單可捲動（8 個都能選）、時代徵兆放在清單外、右側面板 y=62～640、祈禱卡精簡成一行（選取後展開）、神格與模式卡文字 18～22px、第一次評定會延到第 1 年秋天、開局「屆時」預估（engaged 23 局各區間誤差 ≦13pt）。</t>
   </si>
   <si>
+    <t>v0.9c / 視覚100%</t>
+  </si>
+  <si>
+    <t>視覚チームの納品ドット（人物・魔物・建物・地面タイル・小物・樹木・戦闘画面）をゲームに組み込み。画面は実 1280×720、カメラ倍率 ×1／×1.5／×2（ホイール・＋／−キー）。×1 は 48px 版、×2 は _hd 版を 1:1 で表示。老人・子供の補画に残っていた背景色は変換時に除去。夜の窓明かりは納品にライトマスクが無いため一時停止。</t>
+  </si>
+  <si>
+    <t>把視覺團隊交付的點陣圖（人物、魔物、建築、地面 tile、小物件、樹木、戰鬥畫面）接進遊戲。畫面改為實際 1280×720，鏡頭倍率 ×1／×1.5／×2（滾輪、＋／−鍵）。×1 用 48px 版、×2 用 _hd 版 1:1 顯示。老人、小孩補畫殘留的底色在轉換時去除。夜間窗光因交付沒有光照遮罩，暫停。</t>
+  </si>
+  <si>
     <t>V4 攻防・評定会 / V4 攻防與評定會</t>
   </si>
   <si>
@@ -3537,6 +3546,15 @@
   </si>
   <si>
     <t>祈禱清單捲動、時代徵兆位置、右側面板高度、一行祈禱卡、卡片字級、評定會時機（第 1 年秋天）、開局預估重新校準。</t>
+  </si>
+  <si>
+    <t>視覚100% 組み込み</t>
+  </si>
+  <si>
+    <t>人物・魔物・戦闘：納品スプライト。建物26種（冬版あり）、地面タイル4変化＋季節、水辺・崖上は47ブロブ接続、小物35種、樹木4種（季節）。カメラ ×1／×1.5／×2。</t>
+  </si>
+  <si>
+    <t>人物、魔物、戰鬥：交付 sprite。建築 26 種（含冬季版）、地面 tile 4 種變化＋季節、水邊與崖上用 47 blob 拼接、小物件 35 種、樹木 4 種（季節）。鏡頭 ×1／×1.5／×2。</t>
   </si>
 </sst>
 </file>
@@ -7214,7 +7232,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -7378,6 +7396,17 @@
       </c>
       <c r="C16" s="11" t="s">
         <v>1057</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>1060</v>
       </c>
     </row>
   </sheetData>
@@ -7397,24 +7426,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1058</v>
+        <v>1061</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7430,156 +7459,156 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1060</v>
+        <v>1063</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1061</v>
+        <v>1064</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1062</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1063</v>
+        <v>1066</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1064</v>
+        <v>1067</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1065</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1066</v>
+        <v>1069</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1067</v>
+        <v>1070</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1069</v>
+        <v>1072</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1070</v>
+        <v>1073</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1071</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1072</v>
+        <v>1075</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1073</v>
+        <v>1076</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1074</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1077</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1079</v>
+        <v>1082</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1080</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1083</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1085</v>
+        <v>1088</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1086</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1087</v>
+        <v>1090</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1092</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>1093</v>
+        <v>1096</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1094</v>
+        <v>1097</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>1095</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>1098</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>1100</v>
+        <v>1103</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
     </row>
   </sheetData>
@@ -7599,24 +7628,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7632,123 +7661,123 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
     </row>
   </sheetData>
@@ -7891,7 +7920,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -7900,24 +7929,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -7933,123 +7962,134 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1139</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1154</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>1155</v>
+        <v>1158</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>1159</v>
+        <v>1162</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1160</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>1161</v>
+        <v>1164</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>1162</v>
+        <v>1165</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1163</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>1165</v>
+        <v>1168</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>1166</v>
+        <v>1169</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1167</v>
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>1173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>